<commit_message>
update moras y subo documento sprint 7
</commit_message>
<xml_diff>
--- a/Moras BOF.xlsx
+++ b/Moras BOF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ninan\OneDrive\Documentos\Escritorio\UVG\V SEMESTRE\Ingeniería de Software I y II\BOF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E03449FC-FA53-4984-9665-E9A2A3F9FD5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{713306F6-49CA-47B2-B183-A1E25FCBE708}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{31E9EA3E-70BA-40AE-AB5D-089DB34FD579}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
   <si>
     <t>Moras BOF</t>
   </si>
@@ -99,6 +99,9 @@
   </si>
   <si>
     <t>Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abner </t>
   </si>
 </sst>
 </file>
@@ -259,7 +262,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -270,15 +273,6 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -291,6 +285,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -632,15 +636,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.2" x14ac:dyDescent="0.6">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
@@ -714,10 +718,10 @@
         <v>0</v>
       </c>
       <c r="E4" s="3">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F4" s="3">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="G4" s="3">
         <v>0</v>
@@ -726,7 +730,7 @@
         <v>10</v>
       </c>
       <c r="K4" s="6">
-        <v>30</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
@@ -739,6 +743,12 @@
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
+      <c r="J5" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="K5" s="6">
+        <v>40</v>
+      </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
@@ -768,7 +778,7 @@
       </c>
       <c r="B8" s="2">
         <f>SUM(B3:G7)</f>
-        <v>110</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
@@ -778,26 +788,26 @@
       <c r="I10" s="1"/>
     </row>
     <row r="12" spans="1:11" ht="33.6" x14ac:dyDescent="0.65">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="15" t="s">
+      <c r="B13" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
       <c r="F13" s="4" t="s">
         <v>19</v>
       </c>
@@ -807,10 +817,10 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="6"/>
-      <c r="B14" s="16"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
       <c r="F14" s="6"/>
       <c r="G14" s="8">
         <f>SUM(F14:F1048576)</f>
@@ -820,1215 +830,1356 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="6"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="12"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="16"/>
       <c r="F15" s="6"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="6"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="12"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="16"/>
       <c r="F16" s="6"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="6"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="12"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="16"/>
       <c r="F17" s="6"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="6"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="12"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="16"/>
       <c r="F18" s="6"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="6"/>
-      <c r="B19" s="10"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="12"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="16"/>
       <c r="F19" s="6"/>
       <c r="G19" s="1"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="6"/>
-      <c r="B20" s="10"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="12"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="16"/>
       <c r="F20" s="6"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
-      <c r="B21" s="10"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="12"/>
+      <c r="B21" s="14"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="16"/>
       <c r="F21" s="6"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="6"/>
-      <c r="B22" s="10"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="12"/>
+      <c r="B22" s="14"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="16"/>
       <c r="F22" s="6"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="6"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="12"/>
+      <c r="B23" s="14"/>
+      <c r="C23" s="15"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="16"/>
       <c r="F23" s="6"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="6"/>
-      <c r="B24" s="10"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="12"/>
+      <c r="B24" s="14"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="16"/>
       <c r="F24" s="6"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="6"/>
-      <c r="B25" s="10"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="12"/>
+      <c r="B25" s="14"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="16"/>
       <c r="F25" s="6"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="6"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="12"/>
+      <c r="B26" s="14"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="16"/>
       <c r="F26" s="6"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="6"/>
-      <c r="B27" s="10"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="12"/>
+      <c r="B27" s="14"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="16"/>
       <c r="F27" s="6"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="6"/>
-      <c r="B28" s="10"/>
-      <c r="C28" s="11"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="12"/>
+      <c r="B28" s="14"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="16"/>
       <c r="F28" s="6"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="6"/>
-      <c r="B29" s="10"/>
-      <c r="C29" s="11"/>
-      <c r="D29" s="11"/>
-      <c r="E29" s="12"/>
+      <c r="B29" s="14"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="16"/>
       <c r="F29" s="6"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="6"/>
-      <c r="B30" s="10"/>
-      <c r="C30" s="11"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="12"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="16"/>
       <c r="F30" s="6"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="6"/>
-      <c r="B31" s="10"/>
-      <c r="C31" s="11"/>
-      <c r="D31" s="11"/>
-      <c r="E31" s="12"/>
+      <c r="B31" s="14"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="16"/>
       <c r="F31" s="6"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="6"/>
-      <c r="B32" s="10"/>
-      <c r="C32" s="11"/>
-      <c r="D32" s="11"/>
-      <c r="E32" s="12"/>
+      <c r="B32" s="14"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="16"/>
       <c r="F32" s="6"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="6"/>
-      <c r="B33" s="10"/>
-      <c r="C33" s="11"/>
-      <c r="D33" s="11"/>
-      <c r="E33" s="12"/>
+      <c r="B33" s="14"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="16"/>
       <c r="F33" s="6"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="6"/>
-      <c r="B34" s="10"/>
-      <c r="C34" s="11"/>
-      <c r="D34" s="11"/>
-      <c r="E34" s="12"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="16"/>
       <c r="F34" s="6"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="6"/>
-      <c r="B35" s="10"/>
-      <c r="C35" s="11"/>
-      <c r="D35" s="11"/>
-      <c r="E35" s="12"/>
+      <c r="B35" s="14"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="16"/>
       <c r="F35" s="6"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="6"/>
-      <c r="B36" s="10"/>
-      <c r="C36" s="11"/>
-      <c r="D36" s="11"/>
-      <c r="E36" s="12"/>
+      <c r="B36" s="14"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="16"/>
       <c r="F36" s="6"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="6"/>
-      <c r="B37" s="10"/>
-      <c r="C37" s="11"/>
-      <c r="D37" s="11"/>
-      <c r="E37" s="12"/>
+      <c r="B37" s="14"/>
+      <c r="C37" s="15"/>
+      <c r="D37" s="15"/>
+      <c r="E37" s="16"/>
       <c r="F37" s="6"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="6"/>
-      <c r="B38" s="10"/>
-      <c r="C38" s="11"/>
-      <c r="D38" s="11"/>
-      <c r="E38" s="12"/>
+      <c r="B38" s="14"/>
+      <c r="C38" s="15"/>
+      <c r="D38" s="15"/>
+      <c r="E38" s="16"/>
       <c r="F38" s="6"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="6"/>
-      <c r="B39" s="10"/>
-      <c r="C39" s="11"/>
-      <c r="D39" s="11"/>
-      <c r="E39" s="12"/>
+      <c r="B39" s="14"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="15"/>
+      <c r="E39" s="16"/>
       <c r="F39" s="6"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="6"/>
-      <c r="B40" s="10"/>
-      <c r="C40" s="11"/>
-      <c r="D40" s="11"/>
-      <c r="E40" s="12"/>
+      <c r="B40" s="14"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="15"/>
+      <c r="E40" s="16"/>
       <c r="F40" s="6"/>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="6"/>
-      <c r="B41" s="10"/>
-      <c r="C41" s="11"/>
-      <c r="D41" s="11"/>
-      <c r="E41" s="12"/>
+      <c r="B41" s="14"/>
+      <c r="C41" s="15"/>
+      <c r="D41" s="15"/>
+      <c r="E41" s="16"/>
       <c r="F41" s="6"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="6"/>
-      <c r="B42" s="10"/>
-      <c r="C42" s="11"/>
-      <c r="D42" s="11"/>
-      <c r="E42" s="12"/>
+      <c r="B42" s="14"/>
+      <c r="C42" s="15"/>
+      <c r="D42" s="15"/>
+      <c r="E42" s="16"/>
       <c r="F42" s="6"/>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="6"/>
-      <c r="B43" s="10"/>
-      <c r="C43" s="11"/>
-      <c r="D43" s="11"/>
-      <c r="E43" s="12"/>
+      <c r="B43" s="14"/>
+      <c r="C43" s="15"/>
+      <c r="D43" s="15"/>
+      <c r="E43" s="16"/>
       <c r="F43" s="6"/>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="6"/>
-      <c r="B44" s="10"/>
-      <c r="C44" s="11"/>
-      <c r="D44" s="11"/>
-      <c r="E44" s="12"/>
+      <c r="B44" s="14"/>
+      <c r="C44" s="15"/>
+      <c r="D44" s="15"/>
+      <c r="E44" s="16"/>
       <c r="F44" s="6"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="6"/>
-      <c r="B45" s="10"/>
-      <c r="C45" s="11"/>
-      <c r="D45" s="11"/>
-      <c r="E45" s="12"/>
+      <c r="B45" s="14"/>
+      <c r="C45" s="15"/>
+      <c r="D45" s="15"/>
+      <c r="E45" s="16"/>
       <c r="F45" s="6"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="6"/>
-      <c r="B46" s="10"/>
-      <c r="C46" s="11"/>
-      <c r="D46" s="11"/>
-      <c r="E46" s="12"/>
+      <c r="B46" s="14"/>
+      <c r="C46" s="15"/>
+      <c r="D46" s="15"/>
+      <c r="E46" s="16"/>
       <c r="F46" s="6"/>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="6"/>
-      <c r="B47" s="10"/>
-      <c r="C47" s="11"/>
-      <c r="D47" s="11"/>
-      <c r="E47" s="12"/>
+      <c r="B47" s="14"/>
+      <c r="C47" s="15"/>
+      <c r="D47" s="15"/>
+      <c r="E47" s="16"/>
       <c r="F47" s="6"/>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="6"/>
-      <c r="B48" s="10"/>
-      <c r="C48" s="11"/>
-      <c r="D48" s="11"/>
-      <c r="E48" s="12"/>
+      <c r="B48" s="14"/>
+      <c r="C48" s="15"/>
+      <c r="D48" s="15"/>
+      <c r="E48" s="16"/>
       <c r="F48" s="6"/>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="6"/>
-      <c r="B49" s="10"/>
-      <c r="C49" s="11"/>
-      <c r="D49" s="11"/>
-      <c r="E49" s="12"/>
+      <c r="B49" s="14"/>
+      <c r="C49" s="15"/>
+      <c r="D49" s="15"/>
+      <c r="E49" s="16"/>
       <c r="F49" s="6"/>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="6"/>
-      <c r="B50" s="10"/>
-      <c r="C50" s="11"/>
-      <c r="D50" s="11"/>
-      <c r="E50" s="12"/>
+      <c r="B50" s="14"/>
+      <c r="C50" s="15"/>
+      <c r="D50" s="15"/>
+      <c r="E50" s="16"/>
       <c r="F50" s="6"/>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="6"/>
-      <c r="B51" s="10"/>
-      <c r="C51" s="11"/>
-      <c r="D51" s="11"/>
-      <c r="E51" s="12"/>
+      <c r="B51" s="14"/>
+      <c r="C51" s="15"/>
+      <c r="D51" s="15"/>
+      <c r="E51" s="16"/>
       <c r="F51" s="6"/>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="6"/>
-      <c r="B52" s="10"/>
-      <c r="C52" s="11"/>
-      <c r="D52" s="11"/>
-      <c r="E52" s="12"/>
+      <c r="B52" s="14"/>
+      <c r="C52" s="15"/>
+      <c r="D52" s="15"/>
+      <c r="E52" s="16"/>
       <c r="F52" s="6"/>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="6"/>
-      <c r="B53" s="10"/>
-      <c r="C53" s="11"/>
-      <c r="D53" s="11"/>
-      <c r="E53" s="12"/>
+      <c r="B53" s="14"/>
+      <c r="C53" s="15"/>
+      <c r="D53" s="15"/>
+      <c r="E53" s="16"/>
       <c r="F53" s="6"/>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="6"/>
-      <c r="B54" s="10"/>
-      <c r="C54" s="11"/>
-      <c r="D54" s="11"/>
-      <c r="E54" s="12"/>
+      <c r="B54" s="14"/>
+      <c r="C54" s="15"/>
+      <c r="D54" s="15"/>
+      <c r="E54" s="16"/>
       <c r="F54" s="6"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" s="6"/>
-      <c r="B55" s="10"/>
-      <c r="C55" s="11"/>
-      <c r="D55" s="11"/>
-      <c r="E55" s="12"/>
+      <c r="B55" s="14"/>
+      <c r="C55" s="15"/>
+      <c r="D55" s="15"/>
+      <c r="E55" s="16"/>
       <c r="F55" s="6"/>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" s="6"/>
-      <c r="B56" s="10"/>
-      <c r="C56" s="11"/>
-      <c r="D56" s="11"/>
-      <c r="E56" s="12"/>
+      <c r="B56" s="14"/>
+      <c r="C56" s="15"/>
+      <c r="D56" s="15"/>
+      <c r="E56" s="16"/>
       <c r="F56" s="6"/>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="6"/>
-      <c r="B57" s="10"/>
-      <c r="C57" s="11"/>
-      <c r="D57" s="11"/>
-      <c r="E57" s="12"/>
+      <c r="B57" s="14"/>
+      <c r="C57" s="15"/>
+      <c r="D57" s="15"/>
+      <c r="E57" s="16"/>
       <c r="F57" s="6"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="6"/>
-      <c r="B58" s="10"/>
-      <c r="C58" s="11"/>
-      <c r="D58" s="11"/>
-      <c r="E58" s="12"/>
+      <c r="B58" s="14"/>
+      <c r="C58" s="15"/>
+      <c r="D58" s="15"/>
+      <c r="E58" s="16"/>
       <c r="F58" s="6"/>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" s="6"/>
-      <c r="B59" s="10"/>
-      <c r="C59" s="11"/>
-      <c r="D59" s="11"/>
-      <c r="E59" s="12"/>
+      <c r="B59" s="14"/>
+      <c r="C59" s="15"/>
+      <c r="D59" s="15"/>
+      <c r="E59" s="16"/>
       <c r="F59" s="6"/>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" s="6"/>
-      <c r="B60" s="10"/>
-      <c r="C60" s="11"/>
-      <c r="D60" s="11"/>
-      <c r="E60" s="12"/>
+      <c r="B60" s="14"/>
+      <c r="C60" s="15"/>
+      <c r="D60" s="15"/>
+      <c r="E60" s="16"/>
       <c r="F60" s="6"/>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" s="6"/>
-      <c r="B61" s="10"/>
-      <c r="C61" s="11"/>
-      <c r="D61" s="11"/>
-      <c r="E61" s="12"/>
+      <c r="B61" s="14"/>
+      <c r="C61" s="15"/>
+      <c r="D61" s="15"/>
+      <c r="E61" s="16"/>
       <c r="F61" s="6"/>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" s="6"/>
-      <c r="B62" s="10"/>
-      <c r="C62" s="11"/>
-      <c r="D62" s="11"/>
-      <c r="E62" s="12"/>
+      <c r="B62" s="14"/>
+      <c r="C62" s="15"/>
+      <c r="D62" s="15"/>
+      <c r="E62" s="16"/>
       <c r="F62" s="6"/>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" s="6"/>
-      <c r="B63" s="10"/>
-      <c r="C63" s="11"/>
-      <c r="D63" s="11"/>
-      <c r="E63" s="12"/>
+      <c r="B63" s="14"/>
+      <c r="C63" s="15"/>
+      <c r="D63" s="15"/>
+      <c r="E63" s="16"/>
       <c r="F63" s="6"/>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" s="6"/>
-      <c r="B64" s="10"/>
-      <c r="C64" s="11"/>
-      <c r="D64" s="11"/>
-      <c r="E64" s="12"/>
+      <c r="B64" s="14"/>
+      <c r="C64" s="15"/>
+      <c r="D64" s="15"/>
+      <c r="E64" s="16"/>
       <c r="F64" s="6"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" s="6"/>
-      <c r="B65" s="10"/>
-      <c r="C65" s="11"/>
-      <c r="D65" s="11"/>
-      <c r="E65" s="12"/>
+      <c r="B65" s="14"/>
+      <c r="C65" s="15"/>
+      <c r="D65" s="15"/>
+      <c r="E65" s="16"/>
       <c r="F65" s="6"/>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" s="6"/>
-      <c r="B66" s="10"/>
-      <c r="C66" s="11"/>
-      <c r="D66" s="11"/>
-      <c r="E66" s="12"/>
+      <c r="B66" s="14"/>
+      <c r="C66" s="15"/>
+      <c r="D66" s="15"/>
+      <c r="E66" s="16"/>
       <c r="F66" s="6"/>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" s="6"/>
-      <c r="B67" s="10"/>
-      <c r="C67" s="11"/>
-      <c r="D67" s="11"/>
-      <c r="E67" s="12"/>
+      <c r="B67" s="14"/>
+      <c r="C67" s="15"/>
+      <c r="D67" s="15"/>
+      <c r="E67" s="16"/>
       <c r="F67" s="6"/>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" s="6"/>
-      <c r="B68" s="10"/>
-      <c r="C68" s="11"/>
-      <c r="D68" s="11"/>
-      <c r="E68" s="12"/>
+      <c r="B68" s="14"/>
+      <c r="C68" s="15"/>
+      <c r="D68" s="15"/>
+      <c r="E68" s="16"/>
       <c r="F68" s="6"/>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" s="6"/>
-      <c r="B69" s="10"/>
-      <c r="C69" s="11"/>
-      <c r="D69" s="11"/>
-      <c r="E69" s="12"/>
+      <c r="B69" s="14"/>
+      <c r="C69" s="15"/>
+      <c r="D69" s="15"/>
+      <c r="E69" s="16"/>
       <c r="F69" s="6"/>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" s="6"/>
-      <c r="B70" s="10"/>
-      <c r="C70" s="11"/>
-      <c r="D70" s="11"/>
-      <c r="E70" s="12"/>
+      <c r="B70" s="14"/>
+      <c r="C70" s="15"/>
+      <c r="D70" s="15"/>
+      <c r="E70" s="16"/>
       <c r="F70" s="6"/>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" s="6"/>
-      <c r="B71" s="10"/>
-      <c r="C71" s="11"/>
-      <c r="D71" s="11"/>
-      <c r="E71" s="12"/>
+      <c r="B71" s="14"/>
+      <c r="C71" s="15"/>
+      <c r="D71" s="15"/>
+      <c r="E71" s="16"/>
       <c r="F71" s="6"/>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" s="6"/>
-      <c r="B72" s="10"/>
-      <c r="C72" s="11"/>
-      <c r="D72" s="11"/>
-      <c r="E72" s="12"/>
+      <c r="B72" s="14"/>
+      <c r="C72" s="15"/>
+      <c r="D72" s="15"/>
+      <c r="E72" s="16"/>
       <c r="F72" s="6"/>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" s="6"/>
-      <c r="B73" s="10"/>
-      <c r="C73" s="11"/>
-      <c r="D73" s="11"/>
-      <c r="E73" s="12"/>
+      <c r="B73" s="14"/>
+      <c r="C73" s="15"/>
+      <c r="D73" s="15"/>
+      <c r="E73" s="16"/>
       <c r="F73" s="6"/>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" s="6"/>
-      <c r="B74" s="10"/>
-      <c r="C74" s="11"/>
-      <c r="D74" s="11"/>
-      <c r="E74" s="12"/>
+      <c r="B74" s="14"/>
+      <c r="C74" s="15"/>
+      <c r="D74" s="15"/>
+      <c r="E74" s="16"/>
       <c r="F74" s="6"/>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" s="6"/>
-      <c r="B75" s="10"/>
-      <c r="C75" s="11"/>
-      <c r="D75" s="11"/>
-      <c r="E75" s="12"/>
+      <c r="B75" s="14"/>
+      <c r="C75" s="15"/>
+      <c r="D75" s="15"/>
+      <c r="E75" s="16"/>
       <c r="F75" s="6"/>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" s="6"/>
-      <c r="B76" s="10"/>
-      <c r="C76" s="11"/>
-      <c r="D76" s="11"/>
-      <c r="E76" s="12"/>
+      <c r="B76" s="14"/>
+      <c r="C76" s="15"/>
+      <c r="D76" s="15"/>
+      <c r="E76" s="16"/>
       <c r="F76" s="6"/>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" s="6"/>
-      <c r="B77" s="10"/>
-      <c r="C77" s="11"/>
-      <c r="D77" s="11"/>
-      <c r="E77" s="12"/>
+      <c r="B77" s="14"/>
+      <c r="C77" s="15"/>
+      <c r="D77" s="15"/>
+      <c r="E77" s="16"/>
       <c r="F77" s="6"/>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" s="6"/>
-      <c r="B78" s="10"/>
-      <c r="C78" s="11"/>
-      <c r="D78" s="11"/>
-      <c r="E78" s="12"/>
+      <c r="B78" s="14"/>
+      <c r="C78" s="15"/>
+      <c r="D78" s="15"/>
+      <c r="E78" s="16"/>
       <c r="F78" s="6"/>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" s="6"/>
-      <c r="B79" s="10"/>
-      <c r="C79" s="11"/>
-      <c r="D79" s="11"/>
-      <c r="E79" s="12"/>
+      <c r="B79" s="14"/>
+      <c r="C79" s="15"/>
+      <c r="D79" s="15"/>
+      <c r="E79" s="16"/>
       <c r="F79" s="6"/>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" s="6"/>
-      <c r="B80" s="10"/>
-      <c r="C80" s="11"/>
-      <c r="D80" s="11"/>
-      <c r="E80" s="12"/>
+      <c r="B80" s="14"/>
+      <c r="C80" s="15"/>
+      <c r="D80" s="15"/>
+      <c r="E80" s="16"/>
       <c r="F80" s="6"/>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" s="6"/>
-      <c r="B81" s="10"/>
-      <c r="C81" s="11"/>
-      <c r="D81" s="11"/>
-      <c r="E81" s="12"/>
+      <c r="B81" s="14"/>
+      <c r="C81" s="15"/>
+      <c r="D81" s="15"/>
+      <c r="E81" s="16"/>
       <c r="F81" s="6"/>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" s="6"/>
-      <c r="B82" s="10"/>
-      <c r="C82" s="11"/>
-      <c r="D82" s="11"/>
-      <c r="E82" s="12"/>
+      <c r="B82" s="14"/>
+      <c r="C82" s="15"/>
+      <c r="D82" s="15"/>
+      <c r="E82" s="16"/>
       <c r="F82" s="6"/>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" s="6"/>
-      <c r="B83" s="10"/>
-      <c r="C83" s="11"/>
-      <c r="D83" s="11"/>
-      <c r="E83" s="12"/>
+      <c r="B83" s="14"/>
+      <c r="C83" s="15"/>
+      <c r="D83" s="15"/>
+      <c r="E83" s="16"/>
       <c r="F83" s="6"/>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" s="6"/>
-      <c r="B84" s="10"/>
-      <c r="C84" s="11"/>
-      <c r="D84" s="11"/>
-      <c r="E84" s="12"/>
+      <c r="B84" s="14"/>
+      <c r="C84" s="15"/>
+      <c r="D84" s="15"/>
+      <c r="E84" s="16"/>
       <c r="F84" s="6"/>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" s="6"/>
-      <c r="B85" s="10"/>
-      <c r="C85" s="11"/>
-      <c r="D85" s="11"/>
-      <c r="E85" s="12"/>
+      <c r="B85" s="14"/>
+      <c r="C85" s="15"/>
+      <c r="D85" s="15"/>
+      <c r="E85" s="16"/>
       <c r="F85" s="6"/>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" s="6"/>
-      <c r="B86" s="10"/>
-      <c r="C86" s="11"/>
-      <c r="D86" s="11"/>
-      <c r="E86" s="12"/>
+      <c r="B86" s="14"/>
+      <c r="C86" s="15"/>
+      <c r="D86" s="15"/>
+      <c r="E86" s="16"/>
       <c r="F86" s="6"/>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" s="6"/>
-      <c r="B87" s="10"/>
-      <c r="C87" s="11"/>
-      <c r="D87" s="11"/>
-      <c r="E87" s="12"/>
+      <c r="B87" s="14"/>
+      <c r="C87" s="15"/>
+      <c r="D87" s="15"/>
+      <c r="E87" s="16"/>
       <c r="F87" s="6"/>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" s="6"/>
-      <c r="B88" s="10"/>
-      <c r="C88" s="11"/>
-      <c r="D88" s="11"/>
-      <c r="E88" s="12"/>
+      <c r="B88" s="14"/>
+      <c r="C88" s="15"/>
+      <c r="D88" s="15"/>
+      <c r="E88" s="16"/>
       <c r="F88" s="6"/>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" s="6"/>
-      <c r="B89" s="10"/>
-      <c r="C89" s="11"/>
-      <c r="D89" s="11"/>
-      <c r="E89" s="12"/>
+      <c r="B89" s="14"/>
+      <c r="C89" s="15"/>
+      <c r="D89" s="15"/>
+      <c r="E89" s="16"/>
       <c r="F89" s="6"/>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" s="6"/>
-      <c r="B90" s="10"/>
-      <c r="C90" s="11"/>
-      <c r="D90" s="11"/>
-      <c r="E90" s="12"/>
+      <c r="B90" s="14"/>
+      <c r="C90" s="15"/>
+      <c r="D90" s="15"/>
+      <c r="E90" s="16"/>
       <c r="F90" s="6"/>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" s="6"/>
-      <c r="B91" s="10"/>
-      <c r="C91" s="11"/>
-      <c r="D91" s="11"/>
-      <c r="E91" s="12"/>
+      <c r="B91" s="14"/>
+      <c r="C91" s="15"/>
+      <c r="D91" s="15"/>
+      <c r="E91" s="16"/>
       <c r="F91" s="6"/>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" s="6"/>
-      <c r="B92" s="10"/>
-      <c r="C92" s="11"/>
-      <c r="D92" s="11"/>
-      <c r="E92" s="12"/>
+      <c r="B92" s="14"/>
+      <c r="C92" s="15"/>
+      <c r="D92" s="15"/>
+      <c r="E92" s="16"/>
       <c r="F92" s="6"/>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" s="6"/>
-      <c r="B93" s="10"/>
-      <c r="C93" s="11"/>
-      <c r="D93" s="11"/>
-      <c r="E93" s="12"/>
+      <c r="B93" s="14"/>
+      <c r="C93" s="15"/>
+      <c r="D93" s="15"/>
+      <c r="E93" s="16"/>
       <c r="F93" s="6"/>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" s="6"/>
-      <c r="B94" s="10"/>
-      <c r="C94" s="11"/>
-      <c r="D94" s="11"/>
-      <c r="E94" s="12"/>
+      <c r="B94" s="14"/>
+      <c r="C94" s="15"/>
+      <c r="D94" s="15"/>
+      <c r="E94" s="16"/>
       <c r="F94" s="6"/>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" s="6"/>
-      <c r="B95" s="10"/>
-      <c r="C95" s="11"/>
-      <c r="D95" s="11"/>
-      <c r="E95" s="12"/>
+      <c r="B95" s="14"/>
+      <c r="C95" s="15"/>
+      <c r="D95" s="15"/>
+      <c r="E95" s="16"/>
       <c r="F95" s="6"/>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96" s="6"/>
-      <c r="B96" s="10"/>
-      <c r="C96" s="11"/>
-      <c r="D96" s="11"/>
-      <c r="E96" s="12"/>
+      <c r="B96" s="14"/>
+      <c r="C96" s="15"/>
+      <c r="D96" s="15"/>
+      <c r="E96" s="16"/>
       <c r="F96" s="6"/>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" s="6"/>
-      <c r="B97" s="10"/>
-      <c r="C97" s="11"/>
-      <c r="D97" s="11"/>
-      <c r="E97" s="12"/>
+      <c r="B97" s="14"/>
+      <c r="C97" s="15"/>
+      <c r="D97" s="15"/>
+      <c r="E97" s="16"/>
       <c r="F97" s="6"/>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98" s="6"/>
-      <c r="B98" s="10"/>
-      <c r="C98" s="11"/>
-      <c r="D98" s="11"/>
-      <c r="E98" s="12"/>
+      <c r="B98" s="14"/>
+      <c r="C98" s="15"/>
+      <c r="D98" s="15"/>
+      <c r="E98" s="16"/>
       <c r="F98" s="6"/>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" s="6"/>
-      <c r="B99" s="10"/>
-      <c r="C99" s="11"/>
-      <c r="D99" s="11"/>
-      <c r="E99" s="12"/>
+      <c r="B99" s="14"/>
+      <c r="C99" s="15"/>
+      <c r="D99" s="15"/>
+      <c r="E99" s="16"/>
       <c r="F99" s="6"/>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" s="6"/>
-      <c r="B100" s="10"/>
-      <c r="C100" s="11"/>
-      <c r="D100" s="11"/>
-      <c r="E100" s="12"/>
+      <c r="B100" s="14"/>
+      <c r="C100" s="15"/>
+      <c r="D100" s="15"/>
+      <c r="E100" s="16"/>
       <c r="F100" s="6"/>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101" s="6"/>
-      <c r="B101" s="10"/>
-      <c r="C101" s="11"/>
-      <c r="D101" s="11"/>
-      <c r="E101" s="12"/>
+      <c r="B101" s="14"/>
+      <c r="C101" s="15"/>
+      <c r="D101" s="15"/>
+      <c r="E101" s="16"/>
       <c r="F101" s="6"/>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" s="6"/>
-      <c r="B102" s="10"/>
-      <c r="C102" s="11"/>
-      <c r="D102" s="11"/>
-      <c r="E102" s="12"/>
+      <c r="B102" s="14"/>
+      <c r="C102" s="15"/>
+      <c r="D102" s="15"/>
+      <c r="E102" s="16"/>
       <c r="F102" s="6"/>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103" s="6"/>
-      <c r="B103" s="10"/>
-      <c r="C103" s="11"/>
-      <c r="D103" s="11"/>
-      <c r="E103" s="12"/>
+      <c r="B103" s="14"/>
+      <c r="C103" s="15"/>
+      <c r="D103" s="15"/>
+      <c r="E103" s="16"/>
       <c r="F103" s="6"/>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104" s="6"/>
-      <c r="B104" s="10"/>
-      <c r="C104" s="11"/>
-      <c r="D104" s="11"/>
-      <c r="E104" s="12"/>
+      <c r="B104" s="14"/>
+      <c r="C104" s="15"/>
+      <c r="D104" s="15"/>
+      <c r="E104" s="16"/>
       <c r="F104" s="6"/>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105" s="6"/>
-      <c r="B105" s="10"/>
-      <c r="C105" s="11"/>
-      <c r="D105" s="11"/>
-      <c r="E105" s="12"/>
+      <c r="B105" s="14"/>
+      <c r="C105" s="15"/>
+      <c r="D105" s="15"/>
+      <c r="E105" s="16"/>
       <c r="F105" s="6"/>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A106" s="6"/>
-      <c r="B106" s="10"/>
-      <c r="C106" s="11"/>
-      <c r="D106" s="11"/>
-      <c r="E106" s="12"/>
+      <c r="B106" s="14"/>
+      <c r="C106" s="15"/>
+      <c r="D106" s="15"/>
+      <c r="E106" s="16"/>
       <c r="F106" s="6"/>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A107" s="6"/>
-      <c r="B107" s="10"/>
-      <c r="C107" s="11"/>
-      <c r="D107" s="11"/>
-      <c r="E107" s="12"/>
+      <c r="B107" s="14"/>
+      <c r="C107" s="15"/>
+      <c r="D107" s="15"/>
+      <c r="E107" s="16"/>
       <c r="F107" s="6"/>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A108" s="6"/>
-      <c r="B108" s="10"/>
-      <c r="C108" s="11"/>
-      <c r="D108" s="11"/>
-      <c r="E108" s="12"/>
+      <c r="B108" s="14"/>
+      <c r="C108" s="15"/>
+      <c r="D108" s="15"/>
+      <c r="E108" s="16"/>
       <c r="F108" s="6"/>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A109" s="6"/>
-      <c r="B109" s="10"/>
-      <c r="C109" s="11"/>
-      <c r="D109" s="11"/>
-      <c r="E109" s="12"/>
+      <c r="B109" s="14"/>
+      <c r="C109" s="15"/>
+      <c r="D109" s="15"/>
+      <c r="E109" s="16"/>
       <c r="F109" s="6"/>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110" s="6"/>
-      <c r="B110" s="10"/>
-      <c r="C110" s="11"/>
-      <c r="D110" s="11"/>
-      <c r="E110" s="12"/>
+      <c r="B110" s="14"/>
+      <c r="C110" s="15"/>
+      <c r="D110" s="15"/>
+      <c r="E110" s="16"/>
       <c r="F110" s="6"/>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111" s="6"/>
-      <c r="B111" s="10"/>
-      <c r="C111" s="11"/>
-      <c r="D111" s="11"/>
-      <c r="E111" s="12"/>
+      <c r="B111" s="14"/>
+      <c r="C111" s="15"/>
+      <c r="D111" s="15"/>
+      <c r="E111" s="16"/>
       <c r="F111" s="6"/>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112" s="6"/>
-      <c r="B112" s="10"/>
-      <c r="C112" s="11"/>
-      <c r="D112" s="11"/>
-      <c r="E112" s="12"/>
+      <c r="B112" s="14"/>
+      <c r="C112" s="15"/>
+      <c r="D112" s="15"/>
+      <c r="E112" s="16"/>
       <c r="F112" s="6"/>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A113" s="6"/>
-      <c r="B113" s="10"/>
-      <c r="C113" s="11"/>
-      <c r="D113" s="11"/>
-      <c r="E113" s="12"/>
+      <c r="B113" s="14"/>
+      <c r="C113" s="15"/>
+      <c r="D113" s="15"/>
+      <c r="E113" s="16"/>
       <c r="F113" s="6"/>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114" s="6"/>
-      <c r="B114" s="10"/>
-      <c r="C114" s="11"/>
-      <c r="D114" s="11"/>
-      <c r="E114" s="12"/>
+      <c r="B114" s="14"/>
+      <c r="C114" s="15"/>
+      <c r="D114" s="15"/>
+      <c r="E114" s="16"/>
       <c r="F114" s="6"/>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115" s="6"/>
-      <c r="B115" s="10"/>
-      <c r="C115" s="11"/>
-      <c r="D115" s="11"/>
-      <c r="E115" s="12"/>
+      <c r="B115" s="14"/>
+      <c r="C115" s="15"/>
+      <c r="D115" s="15"/>
+      <c r="E115" s="16"/>
       <c r="F115" s="6"/>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A116" s="6"/>
-      <c r="B116" s="10"/>
-      <c r="C116" s="11"/>
-      <c r="D116" s="11"/>
-      <c r="E116" s="12"/>
+      <c r="B116" s="14"/>
+      <c r="C116" s="15"/>
+      <c r="D116" s="15"/>
+      <c r="E116" s="16"/>
       <c r="F116" s="6"/>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A117" s="6"/>
-      <c r="B117" s="10"/>
-      <c r="C117" s="11"/>
-      <c r="D117" s="11"/>
-      <c r="E117" s="12"/>
+      <c r="B117" s="14"/>
+      <c r="C117" s="15"/>
+      <c r="D117" s="15"/>
+      <c r="E117" s="16"/>
       <c r="F117" s="6"/>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A118" s="6"/>
-      <c r="B118" s="10"/>
-      <c r="C118" s="11"/>
-      <c r="D118" s="11"/>
-      <c r="E118" s="12"/>
+      <c r="B118" s="14"/>
+      <c r="C118" s="15"/>
+      <c r="D118" s="15"/>
+      <c r="E118" s="16"/>
       <c r="F118" s="6"/>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A119" s="6"/>
-      <c r="B119" s="10"/>
-      <c r="C119" s="11"/>
-      <c r="D119" s="11"/>
-      <c r="E119" s="12"/>
+      <c r="B119" s="14"/>
+      <c r="C119" s="15"/>
+      <c r="D119" s="15"/>
+      <c r="E119" s="16"/>
       <c r="F119" s="6"/>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A120" s="6"/>
-      <c r="B120" s="10"/>
-      <c r="C120" s="11"/>
-      <c r="D120" s="11"/>
-      <c r="E120" s="12"/>
+      <c r="B120" s="14"/>
+      <c r="C120" s="15"/>
+      <c r="D120" s="15"/>
+      <c r="E120" s="16"/>
       <c r="F120" s="6"/>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A121" s="6"/>
-      <c r="B121" s="10"/>
-      <c r="C121" s="11"/>
-      <c r="D121" s="11"/>
-      <c r="E121" s="12"/>
+      <c r="B121" s="14"/>
+      <c r="C121" s="15"/>
+      <c r="D121" s="15"/>
+      <c r="E121" s="16"/>
       <c r="F121" s="6"/>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A122" s="6"/>
-      <c r="B122" s="10"/>
-      <c r="C122" s="11"/>
-      <c r="D122" s="11"/>
-      <c r="E122" s="12"/>
+      <c r="B122" s="14"/>
+      <c r="C122" s="15"/>
+      <c r="D122" s="15"/>
+      <c r="E122" s="16"/>
       <c r="F122" s="6"/>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A123" s="6"/>
-      <c r="B123" s="10"/>
-      <c r="C123" s="11"/>
-      <c r="D123" s="11"/>
-      <c r="E123" s="12"/>
+      <c r="B123" s="14"/>
+      <c r="C123" s="15"/>
+      <c r="D123" s="15"/>
+      <c r="E123" s="16"/>
       <c r="F123" s="6"/>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A124" s="6"/>
-      <c r="B124" s="10"/>
-      <c r="C124" s="11"/>
-      <c r="D124" s="11"/>
-      <c r="E124" s="12"/>
+      <c r="B124" s="14"/>
+      <c r="C124" s="15"/>
+      <c r="D124" s="15"/>
+      <c r="E124" s="16"/>
       <c r="F124" s="6"/>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A125" s="6"/>
-      <c r="B125" s="10"/>
-      <c r="C125" s="11"/>
-      <c r="D125" s="11"/>
-      <c r="E125" s="12"/>
+      <c r="B125" s="14"/>
+      <c r="C125" s="15"/>
+      <c r="D125" s="15"/>
+      <c r="E125" s="16"/>
       <c r="F125" s="6"/>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A126" s="6"/>
-      <c r="B126" s="10"/>
-      <c r="C126" s="11"/>
-      <c r="D126" s="11"/>
-      <c r="E126" s="12"/>
+      <c r="B126" s="14"/>
+      <c r="C126" s="15"/>
+      <c r="D126" s="15"/>
+      <c r="E126" s="16"/>
       <c r="F126" s="6"/>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A127" s="6"/>
-      <c r="B127" s="10"/>
-      <c r="C127" s="11"/>
-      <c r="D127" s="11"/>
-      <c r="E127" s="12"/>
+      <c r="B127" s="14"/>
+      <c r="C127" s="15"/>
+      <c r="D127" s="15"/>
+      <c r="E127" s="16"/>
       <c r="F127" s="6"/>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A128" s="6"/>
-      <c r="B128" s="10"/>
-      <c r="C128" s="11"/>
-      <c r="D128" s="11"/>
-      <c r="E128" s="12"/>
+      <c r="B128" s="14"/>
+      <c r="C128" s="15"/>
+      <c r="D128" s="15"/>
+      <c r="E128" s="16"/>
       <c r="F128" s="6"/>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A129" s="6"/>
-      <c r="B129" s="10"/>
-      <c r="C129" s="11"/>
-      <c r="D129" s="11"/>
-      <c r="E129" s="12"/>
+      <c r="B129" s="14"/>
+      <c r="C129" s="15"/>
+      <c r="D129" s="15"/>
+      <c r="E129" s="16"/>
       <c r="F129" s="6"/>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A130" s="6"/>
-      <c r="B130" s="10"/>
-      <c r="C130" s="11"/>
-      <c r="D130" s="11"/>
-      <c r="E130" s="12"/>
+      <c r="B130" s="14"/>
+      <c r="C130" s="15"/>
+      <c r="D130" s="15"/>
+      <c r="E130" s="16"/>
       <c r="F130" s="6"/>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A131" s="6"/>
-      <c r="B131" s="10"/>
-      <c r="C131" s="11"/>
-      <c r="D131" s="11"/>
-      <c r="E131" s="12"/>
+      <c r="B131" s="14"/>
+      <c r="C131" s="15"/>
+      <c r="D131" s="15"/>
+      <c r="E131" s="16"/>
       <c r="F131" s="6"/>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A132" s="6"/>
-      <c r="B132" s="10"/>
-      <c r="C132" s="11"/>
-      <c r="D132" s="11"/>
-      <c r="E132" s="12"/>
+      <c r="B132" s="14"/>
+      <c r="C132" s="15"/>
+      <c r="D132" s="15"/>
+      <c r="E132" s="16"/>
       <c r="F132" s="6"/>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A133" s="6"/>
-      <c r="B133" s="10"/>
-      <c r="C133" s="11"/>
-      <c r="D133" s="11"/>
-      <c r="E133" s="12"/>
+      <c r="B133" s="14"/>
+      <c r="C133" s="15"/>
+      <c r="D133" s="15"/>
+      <c r="E133" s="16"/>
       <c r="F133" s="6"/>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A134" s="6"/>
-      <c r="B134" s="10"/>
-      <c r="C134" s="11"/>
-      <c r="D134" s="11"/>
-      <c r="E134" s="12"/>
+      <c r="B134" s="14"/>
+      <c r="C134" s="15"/>
+      <c r="D134" s="15"/>
+      <c r="E134" s="16"/>
       <c r="F134" s="6"/>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A135" s="6"/>
-      <c r="B135" s="10"/>
-      <c r="C135" s="11"/>
-      <c r="D135" s="11"/>
-      <c r="E135" s="12"/>
+      <c r="B135" s="14"/>
+      <c r="C135" s="15"/>
+      <c r="D135" s="15"/>
+      <c r="E135" s="16"/>
       <c r="F135" s="6"/>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A136" s="6"/>
-      <c r="B136" s="10"/>
-      <c r="C136" s="11"/>
-      <c r="D136" s="11"/>
-      <c r="E136" s="12"/>
+      <c r="B136" s="14"/>
+      <c r="C136" s="15"/>
+      <c r="D136" s="15"/>
+      <c r="E136" s="16"/>
       <c r="F136" s="6"/>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A137" s="6"/>
-      <c r="B137" s="10"/>
-      <c r="C137" s="11"/>
-      <c r="D137" s="11"/>
-      <c r="E137" s="12"/>
+      <c r="B137" s="14"/>
+      <c r="C137" s="15"/>
+      <c r="D137" s="15"/>
+      <c r="E137" s="16"/>
       <c r="F137" s="6"/>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A138" s="6"/>
-      <c r="B138" s="10"/>
-      <c r="C138" s="11"/>
-      <c r="D138" s="11"/>
-      <c r="E138" s="12"/>
+      <c r="B138" s="14"/>
+      <c r="C138" s="15"/>
+      <c r="D138" s="15"/>
+      <c r="E138" s="16"/>
       <c r="F138" s="6"/>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A139" s="6"/>
-      <c r="B139" s="10"/>
-      <c r="C139" s="11"/>
-      <c r="D139" s="11"/>
-      <c r="E139" s="12"/>
+      <c r="B139" s="14"/>
+      <c r="C139" s="15"/>
+      <c r="D139" s="15"/>
+      <c r="E139" s="16"/>
       <c r="F139" s="6"/>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A140" s="6"/>
-      <c r="B140" s="10"/>
-      <c r="C140" s="11"/>
-      <c r="D140" s="11"/>
-      <c r="E140" s="12"/>
+      <c r="B140" s="14"/>
+      <c r="C140" s="15"/>
+      <c r="D140" s="15"/>
+      <c r="E140" s="16"/>
       <c r="F140" s="6"/>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A141" s="6"/>
-      <c r="B141" s="10"/>
-      <c r="C141" s="11"/>
-      <c r="D141" s="11"/>
-      <c r="E141" s="12"/>
+      <c r="B141" s="14"/>
+      <c r="C141" s="15"/>
+      <c r="D141" s="15"/>
+      <c r="E141" s="16"/>
       <c r="F141" s="6"/>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A142" s="6"/>
-      <c r="B142" s="10"/>
-      <c r="C142" s="11"/>
-      <c r="D142" s="11"/>
-      <c r="E142" s="12"/>
+      <c r="B142" s="14"/>
+      <c r="C142" s="15"/>
+      <c r="D142" s="15"/>
+      <c r="E142" s="16"/>
       <c r="F142" s="6"/>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A143" s="6"/>
-      <c r="B143" s="10"/>
-      <c r="C143" s="11"/>
-      <c r="D143" s="11"/>
-      <c r="E143" s="12"/>
+      <c r="B143" s="14"/>
+      <c r="C143" s="15"/>
+      <c r="D143" s="15"/>
+      <c r="E143" s="16"/>
       <c r="F143" s="6"/>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A144" s="6"/>
-      <c r="B144" s="10"/>
-      <c r="C144" s="11"/>
-      <c r="D144" s="11"/>
-      <c r="E144" s="12"/>
+      <c r="B144" s="14"/>
+      <c r="C144" s="15"/>
+      <c r="D144" s="15"/>
+      <c r="E144" s="16"/>
       <c r="F144" s="6"/>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A145" s="6"/>
-      <c r="B145" s="10"/>
-      <c r="C145" s="11"/>
-      <c r="D145" s="11"/>
-      <c r="E145" s="12"/>
+      <c r="B145" s="14"/>
+      <c r="C145" s="15"/>
+      <c r="D145" s="15"/>
+      <c r="E145" s="16"/>
       <c r="F145" s="6"/>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A146" s="6"/>
-      <c r="B146" s="10"/>
-      <c r="C146" s="11"/>
-      <c r="D146" s="11"/>
-      <c r="E146" s="12"/>
+      <c r="B146" s="14"/>
+      <c r="C146" s="15"/>
+      <c r="D146" s="15"/>
+      <c r="E146" s="16"/>
       <c r="F146" s="6"/>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A147" s="6"/>
-      <c r="B147" s="10"/>
-      <c r="C147" s="11"/>
-      <c r="D147" s="11"/>
-      <c r="E147" s="12"/>
+      <c r="B147" s="14"/>
+      <c r="C147" s="15"/>
+      <c r="D147" s="15"/>
+      <c r="E147" s="16"/>
       <c r="F147" s="6"/>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A148" s="6"/>
-      <c r="B148" s="10"/>
-      <c r="C148" s="11"/>
-      <c r="D148" s="11"/>
-      <c r="E148" s="12"/>
+      <c r="B148" s="14"/>
+      <c r="C148" s="15"/>
+      <c r="D148" s="15"/>
+      <c r="E148" s="16"/>
       <c r="F148" s="6"/>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A149" s="6"/>
-      <c r="B149" s="10"/>
-      <c r="C149" s="11"/>
-      <c r="D149" s="11"/>
-      <c r="E149" s="12"/>
+      <c r="B149" s="14"/>
+      <c r="C149" s="15"/>
+      <c r="D149" s="15"/>
+      <c r="E149" s="16"/>
       <c r="F149" s="6"/>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A150" s="6"/>
-      <c r="B150" s="10"/>
-      <c r="C150" s="11"/>
-      <c r="D150" s="11"/>
-      <c r="E150" s="12"/>
+      <c r="B150" s="14"/>
+      <c r="C150" s="15"/>
+      <c r="D150" s="15"/>
+      <c r="E150" s="16"/>
       <c r="F150" s="6"/>
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A151" s="6"/>
-      <c r="B151" s="10"/>
-      <c r="C151" s="11"/>
-      <c r="D151" s="11"/>
-      <c r="E151" s="12"/>
+      <c r="B151" s="14"/>
+      <c r="C151" s="15"/>
+      <c r="D151" s="15"/>
+      <c r="E151" s="16"/>
       <c r="F151" s="6"/>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A152" s="6"/>
-      <c r="B152" s="10"/>
-      <c r="C152" s="11"/>
-      <c r="D152" s="11"/>
-      <c r="E152" s="12"/>
+      <c r="B152" s="14"/>
+      <c r="C152" s="15"/>
+      <c r="D152" s="15"/>
+      <c r="E152" s="16"/>
       <c r="F152" s="6"/>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A153" s="6"/>
-      <c r="B153" s="10"/>
-      <c r="C153" s="11"/>
-      <c r="D153" s="11"/>
-      <c r="E153" s="12"/>
+      <c r="B153" s="14"/>
+      <c r="C153" s="15"/>
+      <c r="D153" s="15"/>
+      <c r="E153" s="16"/>
       <c r="F153" s="6"/>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A154" s="6"/>
-      <c r="B154" s="10"/>
-      <c r="C154" s="11"/>
-      <c r="D154" s="11"/>
-      <c r="E154" s="12"/>
+      <c r="B154" s="14"/>
+      <c r="C154" s="15"/>
+      <c r="D154" s="15"/>
+      <c r="E154" s="16"/>
       <c r="F154" s="6"/>
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A155" s="6"/>
-      <c r="B155" s="10"/>
-      <c r="C155" s="11"/>
-      <c r="D155" s="11"/>
-      <c r="E155" s="12"/>
+      <c r="B155" s="14"/>
+      <c r="C155" s="15"/>
+      <c r="D155" s="15"/>
+      <c r="E155" s="16"/>
       <c r="F155" s="6"/>
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A156" s="6"/>
-      <c r="B156" s="10"/>
-      <c r="C156" s="11"/>
-      <c r="D156" s="11"/>
-      <c r="E156" s="12"/>
+      <c r="B156" s="14"/>
+      <c r="C156" s="15"/>
+      <c r="D156" s="15"/>
+      <c r="E156" s="16"/>
       <c r="F156" s="6"/>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A157" s="6"/>
-      <c r="B157" s="10"/>
-      <c r="C157" s="11"/>
-      <c r="D157" s="11"/>
-      <c r="E157" s="12"/>
+      <c r="B157" s="14"/>
+      <c r="C157" s="15"/>
+      <c r="D157" s="15"/>
+      <c r="E157" s="16"/>
       <c r="F157" s="6"/>
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A158" s="6"/>
-      <c r="B158" s="10"/>
-      <c r="C158" s="11"/>
-      <c r="D158" s="11"/>
-      <c r="E158" s="12"/>
+      <c r="B158" s="14"/>
+      <c r="C158" s="15"/>
+      <c r="D158" s="15"/>
+      <c r="E158" s="16"/>
       <c r="F158" s="6"/>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A159" s="6"/>
-      <c r="B159" s="10"/>
-      <c r="C159" s="11"/>
-      <c r="D159" s="11"/>
-      <c r="E159" s="12"/>
+      <c r="B159" s="14"/>
+      <c r="C159" s="15"/>
+      <c r="D159" s="15"/>
+      <c r="E159" s="16"/>
       <c r="F159" s="6"/>
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A160" s="6"/>
-      <c r="B160" s="10"/>
-      <c r="C160" s="11"/>
-      <c r="D160" s="11"/>
-      <c r="E160" s="12"/>
+      <c r="B160" s="14"/>
+      <c r="C160" s="15"/>
+      <c r="D160" s="15"/>
+      <c r="E160" s="16"/>
       <c r="F160" s="6"/>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A161" s="6"/>
-      <c r="B161" s="10"/>
-      <c r="C161" s="11"/>
-      <c r="D161" s="11"/>
-      <c r="E161" s="12"/>
+      <c r="B161" s="14"/>
+      <c r="C161" s="15"/>
+      <c r="D161" s="15"/>
+      <c r="E161" s="16"/>
       <c r="F161" s="6"/>
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A162" s="6"/>
-      <c r="B162" s="10"/>
-      <c r="C162" s="11"/>
-      <c r="D162" s="11"/>
-      <c r="E162" s="12"/>
+      <c r="B162" s="14"/>
+      <c r="C162" s="15"/>
+      <c r="D162" s="15"/>
+      <c r="E162" s="16"/>
       <c r="F162" s="6"/>
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A163" s="6"/>
-      <c r="B163" s="10"/>
-      <c r="C163" s="11"/>
-      <c r="D163" s="11"/>
-      <c r="E163" s="12"/>
+      <c r="B163" s="14"/>
+      <c r="C163" s="15"/>
+      <c r="D163" s="15"/>
+      <c r="E163" s="16"/>
       <c r="F163" s="6"/>
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A164" s="6"/>
-      <c r="B164" s="10"/>
-      <c r="C164" s="11"/>
-      <c r="D164" s="11"/>
-      <c r="E164" s="12"/>
+      <c r="B164" s="14"/>
+      <c r="C164" s="15"/>
+      <c r="D164" s="15"/>
+      <c r="E164" s="16"/>
       <c r="F164" s="6"/>
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A165" s="6"/>
-      <c r="B165" s="10"/>
-      <c r="C165" s="11"/>
-      <c r="D165" s="11"/>
-      <c r="E165" s="12"/>
+      <c r="B165" s="14"/>
+      <c r="C165" s="15"/>
+      <c r="D165" s="15"/>
+      <c r="E165" s="16"/>
       <c r="F165" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="155">
+    <mergeCell ref="B165:E165"/>
+    <mergeCell ref="B160:E160"/>
+    <mergeCell ref="B161:E161"/>
+    <mergeCell ref="B162:E162"/>
+    <mergeCell ref="B163:E163"/>
+    <mergeCell ref="B164:E164"/>
+    <mergeCell ref="B155:E155"/>
+    <mergeCell ref="B156:E156"/>
+    <mergeCell ref="B157:E157"/>
+    <mergeCell ref="B158:E158"/>
+    <mergeCell ref="B159:E159"/>
+    <mergeCell ref="B150:E150"/>
+    <mergeCell ref="B151:E151"/>
+    <mergeCell ref="B152:E152"/>
+    <mergeCell ref="B153:E153"/>
+    <mergeCell ref="B154:E154"/>
+    <mergeCell ref="B145:E145"/>
+    <mergeCell ref="B146:E146"/>
+    <mergeCell ref="B147:E147"/>
+    <mergeCell ref="B148:E148"/>
+    <mergeCell ref="B149:E149"/>
+    <mergeCell ref="B140:E140"/>
+    <mergeCell ref="B141:E141"/>
+    <mergeCell ref="B142:E142"/>
+    <mergeCell ref="B143:E143"/>
+    <mergeCell ref="B144:E144"/>
+    <mergeCell ref="B135:E135"/>
+    <mergeCell ref="B136:E136"/>
+    <mergeCell ref="B137:E137"/>
+    <mergeCell ref="B138:E138"/>
+    <mergeCell ref="B139:E139"/>
+    <mergeCell ref="B130:E130"/>
+    <mergeCell ref="B131:E131"/>
+    <mergeCell ref="B132:E132"/>
+    <mergeCell ref="B133:E133"/>
+    <mergeCell ref="B134:E134"/>
+    <mergeCell ref="B125:E125"/>
+    <mergeCell ref="B126:E126"/>
+    <mergeCell ref="B127:E127"/>
+    <mergeCell ref="B128:E128"/>
+    <mergeCell ref="B129:E129"/>
+    <mergeCell ref="B120:E120"/>
+    <mergeCell ref="B121:E121"/>
+    <mergeCell ref="B122:E122"/>
+    <mergeCell ref="B123:E123"/>
+    <mergeCell ref="B124:E124"/>
+    <mergeCell ref="B115:E115"/>
+    <mergeCell ref="B116:E116"/>
+    <mergeCell ref="B117:E117"/>
+    <mergeCell ref="B118:E118"/>
+    <mergeCell ref="B119:E119"/>
+    <mergeCell ref="B110:E110"/>
+    <mergeCell ref="B111:E111"/>
+    <mergeCell ref="B112:E112"/>
+    <mergeCell ref="B113:E113"/>
+    <mergeCell ref="B114:E114"/>
+    <mergeCell ref="B105:E105"/>
+    <mergeCell ref="B106:E106"/>
+    <mergeCell ref="B107:E107"/>
+    <mergeCell ref="B108:E108"/>
+    <mergeCell ref="B109:E109"/>
+    <mergeCell ref="B100:E100"/>
+    <mergeCell ref="B101:E101"/>
+    <mergeCell ref="B102:E102"/>
+    <mergeCell ref="B103:E103"/>
+    <mergeCell ref="B104:E104"/>
+    <mergeCell ref="B95:E95"/>
+    <mergeCell ref="B96:E96"/>
+    <mergeCell ref="B97:E97"/>
+    <mergeCell ref="B98:E98"/>
+    <mergeCell ref="B99:E99"/>
+    <mergeCell ref="B90:E90"/>
+    <mergeCell ref="B91:E91"/>
+    <mergeCell ref="B92:E92"/>
+    <mergeCell ref="B93:E93"/>
+    <mergeCell ref="B94:E94"/>
+    <mergeCell ref="B85:E85"/>
+    <mergeCell ref="B86:E86"/>
+    <mergeCell ref="B87:E87"/>
+    <mergeCell ref="B88:E88"/>
+    <mergeCell ref="B89:E89"/>
+    <mergeCell ref="B80:E80"/>
+    <mergeCell ref="B81:E81"/>
+    <mergeCell ref="B82:E82"/>
+    <mergeCell ref="B83:E83"/>
+    <mergeCell ref="B84:E84"/>
+    <mergeCell ref="B75:E75"/>
+    <mergeCell ref="B76:E76"/>
+    <mergeCell ref="B77:E77"/>
+    <mergeCell ref="B78:E78"/>
+    <mergeCell ref="B79:E79"/>
+    <mergeCell ref="B70:E70"/>
+    <mergeCell ref="B71:E71"/>
+    <mergeCell ref="B72:E72"/>
+    <mergeCell ref="B73:E73"/>
+    <mergeCell ref="B74:E74"/>
+    <mergeCell ref="B65:E65"/>
+    <mergeCell ref="B66:E66"/>
+    <mergeCell ref="B67:E67"/>
+    <mergeCell ref="B68:E68"/>
+    <mergeCell ref="B69:E69"/>
+    <mergeCell ref="B60:E60"/>
+    <mergeCell ref="B61:E61"/>
+    <mergeCell ref="B62:E62"/>
+    <mergeCell ref="B63:E63"/>
+    <mergeCell ref="B64:E64"/>
+    <mergeCell ref="B55:E55"/>
+    <mergeCell ref="B56:E56"/>
+    <mergeCell ref="B57:E57"/>
+    <mergeCell ref="B58:E58"/>
+    <mergeCell ref="B59:E59"/>
+    <mergeCell ref="B50:E50"/>
+    <mergeCell ref="B51:E51"/>
+    <mergeCell ref="B52:E52"/>
+    <mergeCell ref="B53:E53"/>
+    <mergeCell ref="B54:E54"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="B46:E46"/>
+    <mergeCell ref="B47:E47"/>
+    <mergeCell ref="B48:E48"/>
+    <mergeCell ref="B49:E49"/>
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="B41:E41"/>
+    <mergeCell ref="B42:E42"/>
+    <mergeCell ref="B43:E43"/>
+    <mergeCell ref="B44:E44"/>
+    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="B29:E29"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A12:G12"/>
     <mergeCell ref="B13:E13"/>
@@ -2043,147 +2194,6 @@
     <mergeCell ref="B17:E17"/>
     <mergeCell ref="B18:E18"/>
     <mergeCell ref="B19:E19"/>
-    <mergeCell ref="B30:E30"/>
-    <mergeCell ref="B31:E31"/>
-    <mergeCell ref="B32:E32"/>
-    <mergeCell ref="B33:E33"/>
-    <mergeCell ref="B34:E34"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="B27:E27"/>
-    <mergeCell ref="B28:E28"/>
-    <mergeCell ref="B29:E29"/>
-    <mergeCell ref="B40:E40"/>
-    <mergeCell ref="B41:E41"/>
-    <mergeCell ref="B42:E42"/>
-    <mergeCell ref="B43:E43"/>
-    <mergeCell ref="B44:E44"/>
-    <mergeCell ref="B35:E35"/>
-    <mergeCell ref="B36:E36"/>
-    <mergeCell ref="B37:E37"/>
-    <mergeCell ref="B38:E38"/>
-    <mergeCell ref="B39:E39"/>
-    <mergeCell ref="B50:E50"/>
-    <mergeCell ref="B51:E51"/>
-    <mergeCell ref="B52:E52"/>
-    <mergeCell ref="B53:E53"/>
-    <mergeCell ref="B54:E54"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="B46:E46"/>
-    <mergeCell ref="B47:E47"/>
-    <mergeCell ref="B48:E48"/>
-    <mergeCell ref="B49:E49"/>
-    <mergeCell ref="B60:E60"/>
-    <mergeCell ref="B61:E61"/>
-    <mergeCell ref="B62:E62"/>
-    <mergeCell ref="B63:E63"/>
-    <mergeCell ref="B64:E64"/>
-    <mergeCell ref="B55:E55"/>
-    <mergeCell ref="B56:E56"/>
-    <mergeCell ref="B57:E57"/>
-    <mergeCell ref="B58:E58"/>
-    <mergeCell ref="B59:E59"/>
-    <mergeCell ref="B70:E70"/>
-    <mergeCell ref="B71:E71"/>
-    <mergeCell ref="B72:E72"/>
-    <mergeCell ref="B73:E73"/>
-    <mergeCell ref="B74:E74"/>
-    <mergeCell ref="B65:E65"/>
-    <mergeCell ref="B66:E66"/>
-    <mergeCell ref="B67:E67"/>
-    <mergeCell ref="B68:E68"/>
-    <mergeCell ref="B69:E69"/>
-    <mergeCell ref="B80:E80"/>
-    <mergeCell ref="B81:E81"/>
-    <mergeCell ref="B82:E82"/>
-    <mergeCell ref="B83:E83"/>
-    <mergeCell ref="B84:E84"/>
-    <mergeCell ref="B75:E75"/>
-    <mergeCell ref="B76:E76"/>
-    <mergeCell ref="B77:E77"/>
-    <mergeCell ref="B78:E78"/>
-    <mergeCell ref="B79:E79"/>
-    <mergeCell ref="B90:E90"/>
-    <mergeCell ref="B91:E91"/>
-    <mergeCell ref="B92:E92"/>
-    <mergeCell ref="B93:E93"/>
-    <mergeCell ref="B94:E94"/>
-    <mergeCell ref="B85:E85"/>
-    <mergeCell ref="B86:E86"/>
-    <mergeCell ref="B87:E87"/>
-    <mergeCell ref="B88:E88"/>
-    <mergeCell ref="B89:E89"/>
-    <mergeCell ref="B100:E100"/>
-    <mergeCell ref="B101:E101"/>
-    <mergeCell ref="B102:E102"/>
-    <mergeCell ref="B103:E103"/>
-    <mergeCell ref="B104:E104"/>
-    <mergeCell ref="B95:E95"/>
-    <mergeCell ref="B96:E96"/>
-    <mergeCell ref="B97:E97"/>
-    <mergeCell ref="B98:E98"/>
-    <mergeCell ref="B99:E99"/>
-    <mergeCell ref="B110:E110"/>
-    <mergeCell ref="B111:E111"/>
-    <mergeCell ref="B112:E112"/>
-    <mergeCell ref="B113:E113"/>
-    <mergeCell ref="B114:E114"/>
-    <mergeCell ref="B105:E105"/>
-    <mergeCell ref="B106:E106"/>
-    <mergeCell ref="B107:E107"/>
-    <mergeCell ref="B108:E108"/>
-    <mergeCell ref="B109:E109"/>
-    <mergeCell ref="B120:E120"/>
-    <mergeCell ref="B121:E121"/>
-    <mergeCell ref="B122:E122"/>
-    <mergeCell ref="B123:E123"/>
-    <mergeCell ref="B124:E124"/>
-    <mergeCell ref="B115:E115"/>
-    <mergeCell ref="B116:E116"/>
-    <mergeCell ref="B117:E117"/>
-    <mergeCell ref="B118:E118"/>
-    <mergeCell ref="B119:E119"/>
-    <mergeCell ref="B130:E130"/>
-    <mergeCell ref="B131:E131"/>
-    <mergeCell ref="B132:E132"/>
-    <mergeCell ref="B133:E133"/>
-    <mergeCell ref="B134:E134"/>
-    <mergeCell ref="B125:E125"/>
-    <mergeCell ref="B126:E126"/>
-    <mergeCell ref="B127:E127"/>
-    <mergeCell ref="B128:E128"/>
-    <mergeCell ref="B129:E129"/>
-    <mergeCell ref="B140:E140"/>
-    <mergeCell ref="B141:E141"/>
-    <mergeCell ref="B142:E142"/>
-    <mergeCell ref="B143:E143"/>
-    <mergeCell ref="B144:E144"/>
-    <mergeCell ref="B135:E135"/>
-    <mergeCell ref="B136:E136"/>
-    <mergeCell ref="B137:E137"/>
-    <mergeCell ref="B138:E138"/>
-    <mergeCell ref="B139:E139"/>
-    <mergeCell ref="B150:E150"/>
-    <mergeCell ref="B151:E151"/>
-    <mergeCell ref="B152:E152"/>
-    <mergeCell ref="B153:E153"/>
-    <mergeCell ref="B154:E154"/>
-    <mergeCell ref="B145:E145"/>
-    <mergeCell ref="B146:E146"/>
-    <mergeCell ref="B147:E147"/>
-    <mergeCell ref="B148:E148"/>
-    <mergeCell ref="B149:E149"/>
-    <mergeCell ref="B165:E165"/>
-    <mergeCell ref="B160:E160"/>
-    <mergeCell ref="B161:E161"/>
-    <mergeCell ref="B162:E162"/>
-    <mergeCell ref="B163:E163"/>
-    <mergeCell ref="B164:E164"/>
-    <mergeCell ref="B155:E155"/>
-    <mergeCell ref="B156:E156"/>
-    <mergeCell ref="B157:E157"/>
-    <mergeCell ref="B158:E158"/>
-    <mergeCell ref="B159:E159"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
documentos sprint 9  y update moras
</commit_message>
<xml_diff>
--- a/Moras BOF.xlsx
+++ b/Moras BOF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ninan\OneDrive\Documentos\Escritorio\UVG\V SEMESTRE\Ingeniería de Software I y II\BOF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95F70AA5-1C4E-40F1-9788-1E328374C6B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB502B74-D019-49B7-B877-0A5100863133}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{31E9EA3E-70BA-40AE-AB5D-089DB34FD579}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
   <si>
     <t>Moras BOF</t>
   </si>
@@ -265,7 +265,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -297,6 +297,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -681,7 +682,7 @@
       </c>
       <c r="N2">
         <f>SUM(K3:K8)</f>
-        <v>270</v>
+        <v>380</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
@@ -776,17 +777,29 @@
       <c r="A6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
+      <c r="B6" s="3">
+        <v>110</v>
+      </c>
+      <c r="C6" s="3">
+        <v>20</v>
+      </c>
+      <c r="D6" s="3">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3">
+        <v>0</v>
+      </c>
+      <c r="F6" s="3">
+        <v>0</v>
+      </c>
+      <c r="G6" s="3">
+        <v>110</v>
+      </c>
       <c r="J6" s="6" t="s">
         <v>6</v>
       </c>
       <c r="K6" s="6">
-        <v>40</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
@@ -799,6 +812,12 @@
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
+      <c r="J7" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="K7" s="17">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
@@ -806,7 +825,7 @@
       </c>
       <c r="B8" s="2">
         <f>SUM(B3:G7)</f>
-        <v>710</v>
+        <v>950</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
@@ -814,6 +833,7 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
     </row>
     <row r="12" spans="1:14" ht="33.6" x14ac:dyDescent="0.65">
       <c r="A12" s="14" t="s">

</xml_diff>